<commit_message>
Include module for dynmaic grid access, update InOutmodule for data input, add new excel sheet for curtailment
</commit_message>
<xml_diff>
--- a/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
+++ b/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDD4224-0817-463C-BEDB-66C6056F28F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57E7AA3-82E7-4D3D-87A0-6A931F1FD880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34450" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38160" yWindow="4120" windowWidth="31600" windowHeight="15240" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Parameters" sheetId="121" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="110">
   <si>
     <t>[p.u.]</t>
   </si>
@@ -385,6 +385,15 @@
   </si>
   <si>
     <t>Enable demand side managment</t>
+  </si>
+  <si>
+    <t>Dynamic Grid Acess</t>
+  </si>
+  <si>
+    <t>pEnableDGA</t>
+  </si>
+  <si>
+    <t>Enable dynamic grid acess, allowing for time and locatioan dependend curtailment</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1195,7 @@
   <sheetPr>
     <tabColor rgb="FF008080"/>
   </sheetPr>
-  <dimension ref="B1:H89"/>
+  <dimension ref="B1:H92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.86328125" defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.3984375" style="1" customWidth="1"/>
@@ -1422,7 +1431,6 @@
     </row>
     <row r="28" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B28" s="3"/>
-      <c r="C28"/>
     </row>
     <row r="29" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B29" s="5" t="s">
@@ -1445,7 +1453,6 @@
     </row>
     <row r="31" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
     </row>
     <row r="32" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B32" s="5" t="s">
@@ -1482,20 +1489,18 @@
         <v>105</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="2:6" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="7" t="s">
-        <v>18</v>
-      </c>
+    <row r="37" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B37" s="3"/>
     </row>
     <row r="38" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B38" s="5" t="s">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>24</v>
@@ -1503,21 +1508,23 @@
     </row>
     <row r="39" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B39" s="3" t="s">
-        <v>29</v>
+        <v>108</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="3"/>
+      <c r="F39" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B40" s="7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="41" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B41" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>24</v>
@@ -1525,32 +1532,32 @@
     </row>
     <row r="42" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B42" s="3" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="E42" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="43" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B43" s="3"/>
     </row>
     <row r="44" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B44" s="5" t="s">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>97</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B45" s="3" t="s">
-        <v>98</v>
+        <v>7</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1558,18 +1565,21 @@
     </row>
     <row r="47" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B47" s="5" t="s">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>28</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B48" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C48" s="9">
-        <v>60</v>
+        <v>98</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1577,18 +1587,18 @@
     </row>
     <row r="50" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B50" s="5" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
     </row>
     <row r="51" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B51" s="3" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="C51" s="9">
-        <v>180</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1596,18 +1606,18 @@
     </row>
     <row r="53" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B53" s="5" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B54" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>10</v>
+        <v>50</v>
+      </c>
+      <c r="C54" s="9">
+        <v>180</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1615,21 +1625,18 @@
     </row>
     <row r="56" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B56" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
     </row>
     <row r="57" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B57" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" s="10">
-        <v>0.8</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1637,18 +1644,21 @@
     </row>
     <row r="59" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B59" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>1</v>
+        <v>68</v>
       </c>
     </row>
     <row r="60" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B60" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C60" s="9">
-        <v>1000</v>
+        <v>11</v>
+      </c>
+      <c r="C60" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1656,31 +1666,26 @@
     </row>
     <row r="62" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B62" s="5" t="s">
-        <v>101</v>
+        <v>23</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B63" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="64" spans="2:5" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B64" s="7" t="s">
-        <v>31</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C63" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B64" s="3"/>
     </row>
     <row r="65" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B65" s="5" t="s">
-        <v>32</v>
+        <v>101</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>24</v>
@@ -1688,15 +1693,23 @@
     </row>
     <row r="66" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B66" s="3" t="s">
-        <v>25</v>
+        <v>102</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="E66" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B67" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="68" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B68" s="5" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>24</v>
@@ -1704,52 +1717,39 @@
     </row>
     <row r="69" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B69" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B71" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B72" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C72" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E69" s="1" t="s">
+      <c r="E72" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="71" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B71" s="7" t="s">
+    <row r="74" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B74" s="7" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="72" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B72" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C72" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="73" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B73" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C73" s="10">
-        <v>0</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="74" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B74" s="3"/>
-      <c r="C74"/>
     </row>
     <row r="75" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B75" s="5" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>5</v>
@@ -1757,16 +1757,16 @@
     </row>
     <row r="76" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B76" s="3" t="s">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="C76" s="10">
         <v>0</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G76" s="1" t="s">
         <v>47</v>
@@ -1778,27 +1778,27 @@
     </row>
     <row r="78" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B78" s="5" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B79" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C79" s="13">
-        <v>0.2</v>
+        <v>65</v>
+      </c>
+      <c r="C79" s="10">
+        <v>0</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
     </row>
     <row r="80" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1807,7 +1807,7 @@
     </row>
     <row r="81" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B81" s="5" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>0</v>
@@ -1815,16 +1815,16 @@
     </row>
     <row r="82" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B82" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C82" s="13">
         <v>0.2</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G82" s="1" t="s">
         <v>0</v>
@@ -1834,36 +1834,43 @@
       <c r="B83" s="3"/>
       <c r="C83"/>
     </row>
-    <row r="84" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B84" s="7" t="s">
+    <row r="84" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B84" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B85" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C85" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B86" s="3"/>
+      <c r="C86"/>
+    </row>
+    <row r="87" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B87" s="7" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="85" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B85" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C85" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="86" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B86" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C86" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G86" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="88" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B88" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>70</v>
@@ -1871,15 +1878,37 @@
     </row>
     <row r="89" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B89" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C89" s="10" t="s">
         <v>92</v>
       </c>
       <c r="F89" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B91" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="92" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B92" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C92" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F92" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G89" s="1" t="s">
+      <c r="G92" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1908,7 +1937,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C14:C30 C32:C33 C35:C36">
+  <conditionalFormatting sqref="C14:C27 C29:C30 C32:C33 C35:C36 C38:C39">
     <cfRule type="cellIs" dxfId="31" priority="7" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1916,7 +1945,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C39">
+  <conditionalFormatting sqref="C42">
     <cfRule type="cellIs" dxfId="29" priority="114" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1924,7 +1953,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C42">
+  <conditionalFormatting sqref="C45">
     <cfRule type="cellIs" dxfId="27" priority="92" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1932,7 +1961,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C45">
+  <conditionalFormatting sqref="C48">
     <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1940,7 +1969,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48 C51">
+  <conditionalFormatting sqref="C51 C54">
     <cfRule type="cellIs" dxfId="23" priority="90" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1948,7 +1977,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C54">
+  <conditionalFormatting sqref="C57">
     <cfRule type="cellIs" dxfId="21" priority="88" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1956,7 +1985,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C57">
+  <conditionalFormatting sqref="C60">
     <cfRule type="cellIs" dxfId="19" priority="86" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1964,7 +1993,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C60">
+  <conditionalFormatting sqref="C63">
     <cfRule type="cellIs" dxfId="17" priority="83" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1972,7 +2001,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C63">
+  <conditionalFormatting sqref="C66">
     <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -1980,7 +2009,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C66 C69">
+  <conditionalFormatting sqref="C69 C72">
     <cfRule type="cellIs" dxfId="13" priority="47" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1988,7 +2017,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C73:C74">
+  <conditionalFormatting sqref="C76:C77">
     <cfRule type="cellIs" dxfId="11" priority="97" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -1996,7 +2025,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C76:C77">
+  <conditionalFormatting sqref="C79:C80">
     <cfRule type="cellIs" dxfId="9" priority="36" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -2004,7 +2033,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C79:C80">
+  <conditionalFormatting sqref="C82:C83">
     <cfRule type="cellIs" dxfId="7" priority="31" operator="equal">
       <formula>"No"</formula>
     </cfRule>
@@ -2012,7 +2041,7 @@
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C82:C83">
+  <conditionalFormatting sqref="C85:C86">
     <cfRule type="cellIs" dxfId="5" priority="28" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -2020,7 +2049,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C86">
+  <conditionalFormatting sqref="C89">
     <cfRule type="cellIs" dxfId="3" priority="26" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -2028,7 +2057,7 @@
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C89">
+  <conditionalFormatting sqref="C92">
     <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
@@ -2037,12 +2066,12 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C39 C42 C54 C66 C69 C27 C18 C24 C21 C30:C31 C63 C36 C33" xr:uid="{3037D345-D942-4EE1-9FD6-4C812B603C20}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C42 C45 C57 C69 C72 C27 C18 C24 C21 C36 C66 C33 C39 C30" xr:uid="{3037D345-D942-4EE1-9FD6-4C812B603C20}">
       <formula1>"No, Yes"</formula1>
     </dataValidation>
-    <dataValidation showInputMessage="1" showErrorMessage="1" sqref="C9 C12 C74 C77 C80 C83 C15:C33 C35:C36" xr:uid="{87C6F772-FD4B-9449-B9E7-DA0FF0A031BB}"/>
-    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C73 C57 C76 C79 C82 C86 C89" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C45" xr:uid="{A00608C9-7101-4E98-B005-E178F356E227}">
+    <dataValidation showInputMessage="1" showErrorMessage="1" sqref="C9 C12 C77 C80 C83 C86 C38:C39 C35:C36 C32:C33 C15:C27 C29:C30" xr:uid="{87C6F772-FD4B-9449-B9E7-DA0FF0A031BB}"/>
+    <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="C76 C60 C79 C82 C85 C89 C92" xr:uid="{2B929D69-0393-BA4C-AFD3-02F233DB330E}"/>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C48" xr:uid="{A00608C9-7101-4E98-B005-E178F356E227}">
       <formula1>"NIM,BFM"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2052,12 +2081,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2207,15 +2233,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2239,17 +2276,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Netzknoten Erweiterung in acOpfBfm
DSM mit variabler Netzreduktion in %
Anzeige Variablen werden ausgegeben
</commit_message>
<xml_diff>
--- a/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
+++ b/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tom\Tu Graz\Masterarbeit\Git\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57E7AA3-82E7-4D3D-87A0-6A931F1FD880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215F8082-5C1F-413D-B704-1040E68A46D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38160" yWindow="4120" windowWidth="31600" windowHeight="15240" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Parameters" sheetId="121" r:id="rId1"/>
@@ -43,7 +43,7 @@
     <definedName name="weight_rp">#REF!</definedName>
     <definedName name="zones">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <customWorkbookViews>
     <customWorkbookView name="Andres Ramos - Vista personalizada" guid="{162D0EED-4A71-4EB6-8FDF-A42498BFDBC9}" autoUpdate="1" mergeInterval="5" onlySync="1" personalView="1" maximized="1" windowWidth="1112" windowHeight="624" tabRatio="506" activeSheetId="1"/>
   </customWorkbookViews>
@@ -1196,25 +1196,25 @@
     <tabColor rgb="FF008080"/>
   </sheetPr>
   <dimension ref="B1:H92"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.86328125" defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.3984375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="51" style="1" customWidth="1"/>
-    <col min="3" max="3" width="30.86328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.86328125" style="1"/>
+    <col min="3" max="3" width="30.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="1"/>
     <col min="5" max="5" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="139.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.86328125" style="1"/>
+    <col min="7" max="7" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.21875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:8" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>33</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>34</v>
       </c>
@@ -1250,8 +1250,8 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="7" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
@@ -1276,8 +1276,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="10" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>15</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>3</v>
       </c>
@@ -1302,12 +1302,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:8" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>16</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>27</v>
       </c>
@@ -1332,16 +1332,16 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3"/>
       <c r="C15"/>
     </row>
-    <row r="16" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="5" t="s">
         <v>74</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>75</v>
       </c>
@@ -1360,11 +1360,11 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3"/>
       <c r="C19"/>
     </row>
-    <row r="20" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5" t="s">
         <v>71</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>72</v>
       </c>
@@ -1383,11 +1383,11 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="3"/>
       <c r="C22"/>
     </row>
-    <row r="23" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
         <v>77</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>78</v>
       </c>
@@ -1406,11 +1406,11 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
       <c r="C25"/>
     </row>
-    <row r="26" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>81</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>82</v>
       </c>
@@ -1429,10 +1429,10 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
     </row>
-    <row r="29" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="5" t="s">
         <v>56</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>57</v>
       </c>
@@ -1451,10 +1451,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="5" t="s">
         <v>94</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>93</v>
       </c>
@@ -1473,10 +1473,10 @@
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="3"/>
     </row>
-    <row r="35" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="5" t="s">
         <v>104</v>
       </c>
@@ -1484,21 +1484,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3"/>
     </row>
-    <row r="38" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="5" t="s">
         <v>107</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>108</v>
       </c>
@@ -1517,12 +1517,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="40" spans="2:6" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:6" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="5" t="s">
         <v>19</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>29</v>
       </c>
@@ -1541,10 +1541,10 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="3"/>
     </row>
-    <row r="44" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="5" t="s">
         <v>20</v>
       </c>
@@ -1552,7 +1552,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>7</v>
       </c>
@@ -1560,10 +1560,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3"/>
     </row>
-    <row r="47" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="5" t="s">
         <v>96</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="48" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>98</v>
       </c>
@@ -1582,10 +1582,10 @@
         <v>99</v>
       </c>
     </row>
-    <row r="49" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3"/>
     </row>
-    <row r="50" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="5" t="s">
         <v>21</v>
       </c>
@@ -1593,7 +1593,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>8</v>
       </c>
@@ -1601,10 +1601,10 @@
         <v>60</v>
       </c>
     </row>
-    <row r="52" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="3"/>
     </row>
-    <row r="53" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
         <v>49</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>50</v>
       </c>
@@ -1620,10 +1620,10 @@
         <v>180</v>
       </c>
     </row>
-    <row r="55" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="3"/>
     </row>
-    <row r="56" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="5" t="s">
         <v>67</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>66</v>
       </c>
@@ -1639,10 +1639,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="5" t="s">
         <v>22</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="60" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>11</v>
       </c>
@@ -1661,10 +1661,10 @@
         <v>69</v>
       </c>
     </row>
-    <row r="61" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3"/>
     </row>
-    <row r="62" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="5" t="s">
         <v>23</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>12</v>
       </c>
@@ -1680,10 +1680,10 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="64" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="3"/>
     </row>
-    <row r="65" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="5" t="s">
         <v>101</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>102</v>
       </c>
@@ -1702,12 +1702,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="67" spans="2:7" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:7" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="5" t="s">
         <v>32</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>25</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="5" t="s">
         <v>53</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>54</v>
       </c>
@@ -1742,12 +1742,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="74" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="5" t="s">
         <v>17</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="3" t="s">
         <v>6</v>
       </c>
@@ -1772,11 +1772,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77"/>
     </row>
-    <row r="78" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="5" t="s">
         <v>36</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="3" t="s">
         <v>65</v>
       </c>
@@ -1801,11 +1801,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80"/>
     </row>
-    <row r="81" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="5" t="s">
         <v>59</v>
       </c>
@@ -1813,7 +1813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="3" t="s">
         <v>60</v>
       </c>
@@ -1830,11 +1830,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83"/>
     </row>
-    <row r="84" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="5" t="s">
         <v>36</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="3" t="s">
         <v>62</v>
       </c>
@@ -1859,16 +1859,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86"/>
     </row>
-    <row r="87" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="2:7" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="5" t="s">
         <v>90</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>86</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="5" t="s">
         <v>89</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>88</v>
       </c>

</xml_diff>

<commit_message>
DSM with fixed percentage
Possibility to check in the SQLite of it works or not, and it does :)
</commit_message>
<xml_diff>
--- a/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
+++ b/data/Fertig - 1.a_MS_misch_base/1.a_MS_misch_grid-reduced/Power_Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tom\Tu Graz\Masterarbeit\Git\LEGO-Pyomo\data\Fertig - 1.a_MS_misch_base\1.a_MS_misch_grid-reduced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215F8082-5C1F-413D-B704-1040E68A46D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66726A4F-71E3-4272-93DF-412D74178023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2081,9 +2081,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2233,26 +2236,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2276,9 +2268,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>